<commit_message>
fix: codelijsten relevant unit
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/rie-iepr/rie-iepr.xlsx
+++ b/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/rie-iepr/rie-iepr.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:R34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,72 +407,78 @@
         <v>_type</v>
       </c>
       <c r="C1" t="str">
+        <v>inScheme</v>
+      </c>
+      <c r="D1" t="str">
+        <v>code</v>
+      </c>
+      <c r="E1" t="str">
+        <v>prefLabel</v>
+      </c>
+      <c r="F1" t="str">
+        <v>topConceptOf</v>
+      </c>
+      <c r="G1" t="str">
+        <v>relevantUnit</v>
+      </c>
+      <c r="H1" t="str">
+        <v>relevantDataType</v>
+      </c>
+      <c r="I1" t="str">
+        <v>relevantRiepr</v>
+      </c>
+      <c r="J1" t="str">
         <v>definition</v>
       </c>
-      <c r="D1" t="str">
-        <v>inScheme</v>
-      </c>
-      <c r="E1" t="str">
-        <v>code</v>
-      </c>
-      <c r="F1" t="str">
+      <c r="K1" t="str">
         <v>note</v>
       </c>
-      <c r="G1" t="str">
-        <v>prefLabel</v>
-      </c>
-      <c r="H1" t="str">
-        <v>topConceptOf</v>
-      </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>narrower</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
         <v>narrowerTransitive</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
         <v>semanticRelation</v>
       </c>
-      <c r="L1" t="str">
+      <c r="O1" t="str">
         <v>broader</v>
       </c>
-      <c r="M1" t="str">
+      <c r="P1" t="str">
         <v>broaderTransitive</v>
       </c>
-      <c r="N1" t="str">
+      <c r="Q1" t="str">
         <v>seeAlso</v>
       </c>
-      <c r="O1" t="str">
+      <c r="R1" t="str">
         <v>hasTopConcept</v>
-      </c>
-      <c r="P1" t="str">
-        <v>relevantRiepr</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/emissiepunt</v>
+        <v>http://qudt.org/vocab/unit/M</v>
       </c>
       <c r="B2" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://qudt.org/schema/qudt/Unit|http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C2" t="str">
-        <v>Een regulier emissiepunt.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/eenheden</v>
       </c>
       <c r="D2" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>m</v>
       </c>
       <c r="E2" t="str">
-        <v>emissiepunt</v>
+        <v>Meter</v>
       </c>
       <c r="F2" t="str">
-        <v>Een regulier emissiepunt.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/eenheden</v>
       </c>
       <c r="G2" t="str">
-        <v>Emissiepunt</v>
+        <v>null</v>
       </c>
       <c r="H2" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>null</v>
       </c>
       <c r="I2" t="str">
         <v>null</v>
@@ -496,33 +502,39 @@
         <v>null</v>
       </c>
       <c r="P2" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>null</v>
+      </c>
+      <c r="R2" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/lozingspunt</v>
+        <v>http://qudt.org/vocab/unit/MegaW</v>
       </c>
       <c r="B3" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://qudt.org/schema/qudt/Unit|http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C3" t="str">
-        <v>Een lozing naar water.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/eenheden</v>
       </c>
       <c r="D3" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>MW</v>
       </c>
       <c r="E3" t="str">
-        <v>lozingspunt</v>
+        <v>Mega Watt</v>
       </c>
       <c r="F3" t="str">
-        <v>Een lozing naar water.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/eenheden</v>
       </c>
       <c r="G3" t="str">
-        <v>Lozingspunt</v>
+        <v>null</v>
       </c>
       <c r="H3" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>null</v>
       </c>
       <c r="I3" t="str">
         <v>null</v>
@@ -546,42 +558,48 @@
         <v>null</v>
       </c>
       <c r="P3" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>null</v>
+      </c>
+      <c r="R3" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/schouw-diameter</v>
       </c>
       <c r="B4" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C4" t="str">
-        <v>Een schoorsteen.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
       </c>
       <c r="D4" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>diameter</v>
       </c>
       <c r="E4" t="str">
-        <v>schoorsteen</v>
+        <v>Diameter van de schouw</v>
       </c>
       <c r="F4" t="str">
-        <v>Een schoorsteen.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
       </c>
       <c r="G4" t="str">
-        <v>Schoorsteen</v>
+        <v>http://qudt.org/vocab/unit/M</v>
       </c>
       <c r="H4" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>http://www.w3.org/2001/XMLSchema#decimal</v>
       </c>
       <c r="I4" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schouw</v>
       </c>
       <c r="J4" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom</v>
+        <v>null</v>
       </c>
       <c r="K4" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom</v>
+        <v>null</v>
       </c>
       <c r="L4" t="str">
         <v>null</v>
@@ -596,48 +614,54 @@
         <v>null</v>
       </c>
       <c r="P4" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>null</v>
+      </c>
+      <c r="R4" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/schouw-hoogte</v>
       </c>
       <c r="B5" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C5" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
       </c>
       <c r="D5" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>hoogte</v>
       </c>
       <c r="E5" t="str">
-        <v>schoorsteen_horizontale_uitstroom</v>
+        <v>Hoogte van de schouw</v>
       </c>
       <c r="F5" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
       </c>
       <c r="G5" t="str">
-        <v>Schoorsteen met horizontale uitstroom</v>
+        <v>http://qudt.org/vocab/unit/M</v>
       </c>
       <c r="H5" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>http://www.w3.org/2001/XMLSchema#decimal</v>
       </c>
       <c r="I5" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schouw</v>
       </c>
       <c r="J5" t="str">
         <v>null</v>
       </c>
       <c r="K5" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
+        <v>null</v>
       </c>
       <c r="L5" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
+        <v>null</v>
       </c>
       <c r="M5" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
+        <v>null</v>
       </c>
       <c r="N5" t="str">
         <v>null</v>
@@ -646,48 +670,54 @@
         <v>null</v>
       </c>
       <c r="P5" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>null</v>
+      </c>
+      <c r="R5" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/emissiepunt</v>
       </c>
       <c r="B6" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C6" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="D6" t="str">
+        <v>emissiepunt</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Emissiepunt</v>
+      </c>
+      <c r="F6" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
-      <c r="E6" t="str">
-        <v>schoorsteen_verticale_uitstroom</v>
-      </c>
-      <c r="F6" t="str">
-        <v>null</v>
-      </c>
       <c r="G6" t="str">
-        <v>Schoorsteen met vertikale uitstroom</v>
+        <v>null</v>
       </c>
       <c r="H6" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>null</v>
       </c>
       <c r="I6" t="str">
         <v>null</v>
       </c>
       <c r="J6" t="str">
-        <v>null</v>
+        <v>Een regulier emissiepunt.</v>
       </c>
       <c r="K6" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
+        <v>Een regulier emissiepunt.</v>
       </c>
       <c r="L6" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
+        <v>null</v>
       </c>
       <c r="M6" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
+        <v>null</v>
       </c>
       <c r="N6" t="str">
         <v>null</v>
@@ -696,42 +726,48 @@
         <v>null</v>
       </c>
       <c r="P6" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>null</v>
+      </c>
+      <c r="R6" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schouw</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/lozingspunt</v>
       </c>
       <c r="B7" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C7" t="str">
-        <v>Een schouw.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="D7" t="str">
+        <v>lozingspunt</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Lozingspunt</v>
+      </c>
+      <c r="F7" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
-      <c r="E7" t="str">
-        <v>schouw</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Een schouw.</v>
-      </c>
       <c r="G7" t="str">
-        <v>Schouw</v>
+        <v>null</v>
       </c>
       <c r="H7" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>null</v>
       </c>
       <c r="I7" t="str">
         <v>null</v>
       </c>
       <c r="J7" t="str">
-        <v>null</v>
+        <v>Een lozing naar water.</v>
       </c>
       <c r="K7" t="str">
-        <v>null</v>
+        <v>Een lozing naar water.</v>
       </c>
       <c r="L7" t="str">
         <v>null</v>
@@ -746,92 +782,104 @@
         <v>null</v>
       </c>
       <c r="P7" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>null</v>
+      </c>
+      <c r="R7" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
       </c>
       <c r="B8" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C8" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="D8" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
+        <v>schoorsteen</v>
       </c>
       <c r="E8" t="str">
-        <v>directe_stookinstallatie</v>
+        <v>Schoorsteen</v>
       </c>
       <c r="F8" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="G8" t="str">
-        <v>Directe Stookinstallatie</v>
+        <v>null</v>
       </c>
       <c r="H8" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
+        <v>null</v>
       </c>
       <c r="I8" t="str">
         <v>null</v>
       </c>
       <c r="J8" t="str">
-        <v>null</v>
+        <v>Een schoorsteen.</v>
       </c>
       <c r="K8" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
+        <v>Een schoorsteen.</v>
       </c>
       <c r="L8" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom</v>
       </c>
       <c r="M8" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom</v>
       </c>
       <c r="N8" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom</v>
       </c>
       <c r="O8" t="str">
         <v>null</v>
       </c>
       <c r="P8" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>null</v>
+      </c>
+      <c r="R8" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom</v>
       </c>
       <c r="B9" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C9" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="D9" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
+        <v>schoorsteen_horizontale_uitstroom</v>
       </c>
       <c r="E9" t="str">
-        <v>stookinstallatie</v>
+        <v>Schoorsteen met horizontale uitstroom</v>
       </c>
       <c r="F9" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="G9" t="str">
-        <v>Stookinstallatie</v>
+        <v>null</v>
       </c>
       <c r="H9" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
+        <v>null</v>
       </c>
       <c r="I9" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
+        <v>null</v>
       </c>
       <c r="J9" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
+        <v>null</v>
       </c>
       <c r="K9" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
+        <v>null</v>
       </c>
       <c r="L9" t="str">
         <v>null</v>
@@ -840,39 +888,45 @@
         <v>null</v>
       </c>
       <c r="N9" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
       </c>
       <c r="O9" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
       </c>
       <c r="P9" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>null</v>
+      </c>
+      <c r="R9" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/meetput</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom</v>
       </c>
       <c r="B10" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C10" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="D10" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_type</v>
+        <v>schoorsteen_verticale_uitstroom</v>
       </c>
       <c r="E10" t="str">
-        <v>meetput</v>
+        <v>Schoorsteen met vertikale uitstroom</v>
       </c>
       <c r="F10" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="G10" t="str">
-        <v>Meetput</v>
+        <v>null</v>
       </c>
       <c r="H10" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_type</v>
+        <v>null</v>
       </c>
       <c r="I10" t="str">
         <v>null</v>
@@ -890,48 +944,54 @@
         <v>null</v>
       </c>
       <c r="N10" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
       </c>
       <c r="O10" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
       </c>
       <c r="P10" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>null</v>
+      </c>
+      <c r="R10" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-type/grondwaterput</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schouw</v>
       </c>
       <c r="B11" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C11" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="D11" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_type</v>
+        <v>schouw</v>
       </c>
       <c r="E11" t="str">
-        <v>grondwaterput</v>
+        <v>Schouw</v>
       </c>
       <c r="F11" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="G11" t="str">
-        <v>Grondwaterput</v>
+        <v>null</v>
       </c>
       <c r="H11" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_type</v>
+        <v>null</v>
       </c>
       <c r="I11" t="str">
         <v>null</v>
       </c>
       <c r="J11" t="str">
-        <v>null</v>
+        <v>Een schouw.</v>
       </c>
       <c r="K11" t="str">
-        <v>null</v>
+        <v>Een schouw.</v>
       </c>
       <c r="L11" t="str">
         <v>null</v>
@@ -946,36 +1006,42 @@
         <v>null</v>
       </c>
       <c r="P11" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>null</v>
+      </c>
+      <c r="R11" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/emissie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerd_vermogen</v>
       </c>
       <c r="B12" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C12" t="str">
-        <v>De procedure emissie via een emissiepunt.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_eigenschappen</v>
       </c>
       <c r="D12" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+        <v>GEINSTALLEERD_VERMOGEN</v>
       </c>
       <c r="E12" t="str">
-        <v>EMISSIE</v>
+        <v>Geinstalleerd vermogen</v>
       </c>
       <c r="F12" t="str">
-        <v>De procedure emissie via een emissiepunt.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_eigenschappen</v>
       </c>
       <c r="G12" t="str">
-        <v>Emissie</v>
+        <v>http://qudt.org/vocab/unit/MegaW</v>
       </c>
       <c r="H12" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+        <v>http://www.w3.org/2001/XMLSchema#decimal</v>
       </c>
       <c r="I12" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
       </c>
       <c r="J12" t="str">
         <v>null</v>
@@ -996,33 +1062,39 @@
         <v>null</v>
       </c>
       <c r="P12" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>null</v>
+      </c>
+      <c r="R12" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/onttrekking</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
       </c>
       <c r="B13" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C13" t="str">
-        <v>De procedure onttrekking via een onttrekingspunt.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
       </c>
       <c r="D13" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+        <v>directe_stookinstallatie</v>
       </c>
       <c r="E13" t="str">
-        <v>ONTTREKKING</v>
+        <v>Directe Stookinstallatie</v>
       </c>
       <c r="F13" t="str">
-        <v>De procedure onttrekking via een onttrekingspunt.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
       </c>
       <c r="G13" t="str">
-        <v>Onttrekking</v>
+        <v>null</v>
       </c>
       <c r="H13" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+        <v>null</v>
       </c>
       <c r="I13" t="str">
         <v>null</v>
@@ -1040,39 +1112,45 @@
         <v>null</v>
       </c>
       <c r="N13" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
       </c>
       <c r="O13" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
       </c>
       <c r="P13" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>null</v>
+      </c>
+      <c r="R13" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/transport</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
       </c>
       <c r="B14" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C14" t="str">
-        <v>De procedure transport tussen twee processen.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
       </c>
       <c r="D14" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+        <v>stookinstallatie</v>
       </c>
       <c r="E14" t="str">
-        <v>TRANSPORT</v>
+        <v>Stookinstallatie</v>
       </c>
       <c r="F14" t="str">
-        <v>De procedure transport tussen twee processen.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
       </c>
       <c r="G14" t="str">
-        <v>Transport</v>
+        <v>null</v>
       </c>
       <c r="H14" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+        <v>null</v>
       </c>
       <c r="I14" t="str">
         <v>null</v>
@@ -1084,45 +1162,51 @@
         <v>null</v>
       </c>
       <c r="L14" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
       </c>
       <c r="M14" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
       </c>
       <c r="N14" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
       </c>
       <c r="O14" t="str">
         <v>null</v>
       </c>
       <c r="P14" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>null</v>
+      </c>
+      <c r="R14" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/verwerking</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/meetput</v>
       </c>
       <c r="B15" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C15" t="str">
-        <v>De procedure verwerking door een installatie.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_type</v>
       </c>
       <c r="D15" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+        <v>meetput</v>
       </c>
       <c r="E15" t="str">
-        <v>VERWERKING</v>
+        <v>Meetput</v>
       </c>
       <c r="F15" t="str">
-        <v>De procedure verwerking door een installatie.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_type</v>
       </c>
       <c r="G15" t="str">
-        <v>Verwerking</v>
+        <v>null</v>
       </c>
       <c r="H15" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+        <v>null</v>
       </c>
       <c r="I15" t="str">
         <v>null</v>
@@ -1146,33 +1230,39 @@
         <v>null</v>
       </c>
       <c r="P15" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>null</v>
+      </c>
+      <c r="R15" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/definitief_uit_dienst</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-type/grondwaterput</v>
       </c>
       <c r="B16" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C16" t="str">
-        <v>De status definitief uit dienst geeft aan dat een entiteit definitief buiten gebruik is.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_type</v>
       </c>
       <c r="D16" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>grondwaterput</v>
       </c>
       <c r="E16" t="str">
-        <v>DEFINITIEF_UIT_DIENST</v>
+        <v>Grondwaterput</v>
       </c>
       <c r="F16" t="str">
-        <v>De status definitief uit dienst geeft aan dat een entiteit definitief buiten gebruik is.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_type</v>
       </c>
       <c r="G16" t="str">
-        <v>Definitief uit dienst</v>
+        <v>null</v>
       </c>
       <c r="H16" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>null</v>
       </c>
       <c r="I16" t="str">
         <v>null</v>
@@ -1190,48 +1280,54 @@
         <v>null</v>
       </c>
       <c r="N16" t="str">
-        <v>http://purl.org/adms/status/Withdrawn</v>
+        <v>null</v>
       </c>
       <c r="O16" t="str">
         <v>null</v>
       </c>
       <c r="P16" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>null</v>
+      </c>
+      <c r="R16" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/in_dienst</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/emissie</v>
       </c>
       <c r="B17" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C17" t="str">
-        <v>De status in dienst geeft aan dat een entiteit momenteel in gebruik is.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
       </c>
       <c r="D17" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>EMISSIE</v>
       </c>
       <c r="E17" t="str">
-        <v>IN_DIENST</v>
+        <v>Emissie</v>
       </c>
       <c r="F17" t="str">
-        <v>De status in dienst geeft aan dat een entiteit momenteel in gebruik is.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
       </c>
       <c r="G17" t="str">
-        <v>In dienst</v>
+        <v>null</v>
       </c>
       <c r="H17" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>http://www.w3.org/ns/sosa/Procedure</v>
       </c>
       <c r="I17" t="str">
         <v>null</v>
       </c>
       <c r="J17" t="str">
-        <v>null</v>
+        <v>De procedure emissie via een emissiepunt.</v>
       </c>
       <c r="K17" t="str">
-        <v>null</v>
+        <v>De procedure emissie via een emissiepunt.</v>
       </c>
       <c r="L17" t="str">
         <v>null</v>
@@ -1240,48 +1336,54 @@
         <v>null</v>
       </c>
       <c r="N17" t="str">
-        <v>http://purl.org/adms/status/Completed</v>
+        <v>null</v>
       </c>
       <c r="O17" t="str">
         <v>null</v>
       </c>
       <c r="P17" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>null</v>
+      </c>
+      <c r="R17" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/ontmanteld</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/onttrekking</v>
       </c>
       <c r="B18" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C18" t="str">
-        <v>De status ontmanteld geeft aan dat een entiteit niet meer bestaat.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
       </c>
       <c r="D18" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>ONTTREKKING</v>
       </c>
       <c r="E18" t="str">
-        <v>ONTMANTELD</v>
+        <v>Onttrekking</v>
       </c>
       <c r="F18" t="str">
-        <v>De status ontmanteld geeft aan dat een entiteit niet meer bestaat.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
       </c>
       <c r="G18" t="str">
-        <v>Ontmanteld</v>
+        <v>null</v>
       </c>
       <c r="H18" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>http://www.w3.org/ns/sosa/Procedure</v>
       </c>
       <c r="I18" t="str">
         <v>null</v>
       </c>
       <c r="J18" t="str">
-        <v>null</v>
+        <v>De procedure onttrekking via een onttrekingspunt.</v>
       </c>
       <c r="K18" t="str">
-        <v>null</v>
+        <v>De procedure onttrekking via een onttrekingspunt.</v>
       </c>
       <c r="L18" t="str">
         <v>null</v>
@@ -1290,48 +1392,54 @@
         <v>null</v>
       </c>
       <c r="N18" t="str">
-        <v>http://purl.org/adms/status/Withdrawn</v>
+        <v>null</v>
       </c>
       <c r="O18" t="str">
         <v>null</v>
       </c>
       <c r="P18" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>null</v>
+      </c>
+      <c r="R18" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/tijdelijk_uit_dienst</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/transport</v>
       </c>
       <c r="B19" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C19" t="str">
-        <v>De status tijdelijk uit dienst geeft aan dat een entiteit tijden buiten gebruik is.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
       </c>
       <c r="D19" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>TRANSPORT</v>
       </c>
       <c r="E19" t="str">
-        <v>TIJDELIJK_UIT_DIENST</v>
+        <v>Transport</v>
       </c>
       <c r="F19" t="str">
-        <v>De status tijdelijk uit dienst geeft aan dat een entiteit tijden buiten gebruik is.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
       </c>
       <c r="G19" t="str">
-        <v>Tijdelijk uit dienst</v>
+        <v>null</v>
       </c>
       <c r="H19" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>http://www.w3.org/ns/sosa/Procedure</v>
       </c>
       <c r="I19" t="str">
         <v>null</v>
       </c>
       <c r="J19" t="str">
-        <v>null</v>
+        <v>De procedure transport tussen twee processen.</v>
       </c>
       <c r="K19" t="str">
-        <v>null</v>
+        <v>De procedure transport tussen twee processen.</v>
       </c>
       <c r="L19" t="str">
         <v>null</v>
@@ -1340,48 +1448,54 @@
         <v>null</v>
       </c>
       <c r="N19" t="str">
-        <v>http://purl.org/adms/status/Deprecated</v>
+        <v>null</v>
       </c>
       <c r="O19" t="str">
         <v>null</v>
       </c>
       <c r="P19" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>null</v>
+      </c>
+      <c r="R19" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/voorgesteld</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/verwerking</v>
       </c>
       <c r="B20" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C20" t="str">
-        <v>De status voorgesteld geeft aan dat een entiteit voorsgesteld is door de Vlaamse Overheid.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
       </c>
       <c r="D20" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>VERWERKING</v>
       </c>
       <c r="E20" t="str">
-        <v>VOORGESTELD</v>
+        <v>Verwerking</v>
       </c>
       <c r="F20" t="str">
-        <v>De status voorgesteld geeft aan dat een entiteit voorsgesteld is door de Vlaamse Overheid.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
       </c>
       <c r="G20" t="str">
-        <v>Voorgesteld Ontwerp</v>
+        <v>null</v>
       </c>
       <c r="H20" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>http://www.w3.org/ns/sosa/Procedure</v>
       </c>
       <c r="I20" t="str">
         <v>null</v>
       </c>
       <c r="J20" t="str">
-        <v>null</v>
+        <v>De procedure verwerking door een installatie.</v>
       </c>
       <c r="K20" t="str">
-        <v>null</v>
+        <v>De procedure verwerking door een installatie.</v>
       </c>
       <c r="L20" t="str">
         <v>null</v>
@@ -1390,48 +1504,54 @@
         <v>null</v>
       </c>
       <c r="N20" t="str">
-        <v>http://purl.org/adms/status/UnderDevelopment</v>
+        <v>null</v>
       </c>
       <c r="O20" t="str">
         <v>null</v>
       </c>
       <c r="P20" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>null</v>
+      </c>
+      <c r="R20" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/definitief_uit_dienst</v>
       </c>
       <c r="B21" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C21" t="str">
-        <v>Een typering van verschillende eigenschappen voor emissiepunten.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="D21" t="str">
-        <v>null</v>
+        <v>DEFINITIEF_UIT_DIENST</v>
       </c>
       <c r="E21" t="str">
-        <v>null</v>
+        <v>Definitief uit dienst</v>
       </c>
       <c r="F21" t="str">
-        <v>Een typering van verschillende eigenschappen voor emissiepunten.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="G21" t="str">
-        <v>Emissiepunt eigenschappen</v>
+        <v>null</v>
       </c>
       <c r="H21" t="str">
-        <v>null</v>
+        <v>http://www.w3.org/ns/adms#</v>
       </c>
       <c r="I21" t="str">
         <v>null</v>
       </c>
       <c r="J21" t="str">
-        <v>null</v>
+        <v>De status definitief uit dienst geeft aan dat een entiteit definitief buiten gebruik is.</v>
       </c>
       <c r="K21" t="str">
-        <v>null</v>
+        <v>De status definitief uit dienst geeft aan dat een entiteit definitief buiten gebruik is.</v>
       </c>
       <c r="L21" t="str">
         <v>null</v>
@@ -1443,45 +1563,51 @@
         <v>null</v>
       </c>
       <c r="O21" t="str">
-        <v>riepr-emissiepunt-eigenschappen:schouw-diameter|riepr-emissiepunt-eigenschappen:schouw-hoogte</v>
+        <v>null</v>
       </c>
       <c r="P21" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>http://purl.org/adms/status/Withdrawn</v>
+      </c>
+      <c r="R21" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/in_dienst</v>
       </c>
       <c r="B22" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C22" t="str">
-        <v>Een typering van verschillende soorten emissiepunten.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="D22" t="str">
-        <v>null</v>
+        <v>IN_DIENST</v>
       </c>
       <c r="E22" t="str">
-        <v>null</v>
+        <v>In dienst</v>
       </c>
       <c r="F22" t="str">
-        <v>Een typering van verschillende soorten emissiepunten.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="G22" t="str">
-        <v>Emissiepunt types</v>
+        <v>null</v>
       </c>
       <c r="H22" t="str">
-        <v>null</v>
+        <v>http://www.w3.org/ns/adms#</v>
       </c>
       <c r="I22" t="str">
         <v>null</v>
       </c>
       <c r="J22" t="str">
-        <v>null</v>
+        <v>De status in dienst geeft aan dat een entiteit momenteel in gebruik is.</v>
       </c>
       <c r="K22" t="str">
-        <v>null</v>
+        <v>De status in dienst geeft aan dat een entiteit momenteel in gebruik is.</v>
       </c>
       <c r="L22" t="str">
         <v>null</v>
@@ -1493,45 +1619,51 @@
         <v>null</v>
       </c>
       <c r="O22" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/emissiepunt|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/lozingspunt|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schouw</v>
+        <v>null</v>
       </c>
       <c r="P22" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>http://purl.org/adms/status/Completed</v>
+      </c>
+      <c r="R22" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_eigenschappen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/ontmanteld</v>
       </c>
       <c r="B23" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C23" t="str">
-        <v>Een typering van verschillende eigenschappen voor installaties.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="D23" t="str">
-        <v>null</v>
+        <v>ONTMANTELD</v>
       </c>
       <c r="E23" t="str">
-        <v>null</v>
+        <v>Ontmanteld</v>
       </c>
       <c r="F23" t="str">
-        <v>Een typering van verschillende eigenschappen voor installaties.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="G23" t="str">
-        <v>Installatie eigenschappen</v>
+        <v>null</v>
       </c>
       <c r="H23" t="str">
-        <v>null</v>
+        <v>http://www.w3.org/ns/adms#</v>
       </c>
       <c r="I23" t="str">
         <v>null</v>
       </c>
       <c r="J23" t="str">
-        <v>null</v>
+        <v>De status ontmanteld geeft aan dat een entiteit niet meer bestaat.</v>
       </c>
       <c r="K23" t="str">
-        <v>null</v>
+        <v>De status ontmanteld geeft aan dat een entiteit niet meer bestaat.</v>
       </c>
       <c r="L23" t="str">
         <v>null</v>
@@ -1543,45 +1675,51 @@
         <v>null</v>
       </c>
       <c r="O23" t="str">
-        <v>riepr-installatie-eigenschappen:geinstalleerd_vermogen</v>
+        <v>null</v>
       </c>
       <c r="P23" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>http://purl.org/adms/status/Withdrawn</v>
+      </c>
+      <c r="R23" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/tijdelijk_uit_dienst</v>
       </c>
       <c r="B24" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C24" t="str">
-        <v>Een typering van verschillende soorten installaties.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="D24" t="str">
-        <v>null</v>
+        <v>TIJDELIJK_UIT_DIENST</v>
       </c>
       <c r="E24" t="str">
-        <v>null</v>
+        <v>Tijdelijk uit dienst</v>
       </c>
       <c r="F24" t="str">
-        <v>Een typering van verschillende soorten installaties.</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="G24" t="str">
-        <v>Installatie types</v>
+        <v>null</v>
       </c>
       <c r="H24" t="str">
-        <v>null</v>
+        <v>http://www.w3.org/ns/adms#</v>
       </c>
       <c r="I24" t="str">
         <v>null</v>
       </c>
       <c r="J24" t="str">
-        <v>null</v>
+        <v>De status tijdelijk uit dienst geeft aan dat een entiteit tijden buiten gebruik is.</v>
       </c>
       <c r="K24" t="str">
-        <v>null</v>
+        <v>De status tijdelijk uit dienst geeft aan dat een entiteit tijden buiten gebruik is.</v>
       </c>
       <c r="L24" t="str">
         <v>null</v>
@@ -1593,45 +1731,51 @@
         <v>null</v>
       </c>
       <c r="O24" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
+        <v>null</v>
       </c>
       <c r="P24" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>http://purl.org/adms/status/Deprecated</v>
+      </c>
+      <c r="R24" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_type</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/voorgesteld</v>
       </c>
       <c r="B25" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C25" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="D25" t="str">
-        <v>null</v>
+        <v>VOORGESTELD</v>
       </c>
       <c r="E25" t="str">
-        <v>null</v>
+        <v>Voorgesteld Ontwerp</v>
       </c>
       <c r="F25" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
       </c>
       <c r="G25" t="str">
-        <v>Meetpunt types</v>
+        <v>null</v>
       </c>
       <c r="H25" t="str">
-        <v>null</v>
+        <v>http://www.w3.org/ns/adms#</v>
       </c>
       <c r="I25" t="str">
         <v>null</v>
       </c>
       <c r="J25" t="str">
-        <v>null</v>
+        <v>De status voorgesteld geeft aan dat een entiteit voorsgesteld is door de Vlaamse Overheid.</v>
       </c>
       <c r="K25" t="str">
-        <v>null</v>
+        <v>De status voorgesteld geeft aan dat een entiteit voorsgesteld is door de Vlaamse Overheid.</v>
       </c>
       <c r="L25" t="str">
         <v>null</v>
@@ -1643,21 +1787,27 @@
         <v>null</v>
       </c>
       <c r="O25" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/meetput</v>
+        <v>null</v>
       </c>
       <c r="P25" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>http://purl.org/adms/status/UnderDevelopment</v>
+      </c>
+      <c r="R25" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_type</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/eenheden</v>
       </c>
       <c r="B26" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C26" t="str">
-        <v>Een typering van verschillende soorten onttrekkingspunten.</v>
+        <v>null</v>
       </c>
       <c r="D26" t="str">
         <v>null</v>
@@ -1666,10 +1816,10 @@
         <v>null</v>
       </c>
       <c r="F26" t="str">
-        <v>Een typering van verschillende soorten onttrekkingspunten.</v>
+        <v>null</v>
       </c>
       <c r="G26" t="str">
-        <v>Onttrekkingspunt types</v>
+        <v>null</v>
       </c>
       <c r="H26" t="str">
         <v>null</v>
@@ -1693,33 +1843,39 @@
         <v>null</v>
       </c>
       <c r="O26" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-type/grondwaterput</v>
+        <v>null</v>
       </c>
       <c r="P26" t="str">
         <v>null</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>null</v>
+      </c>
+      <c r="R26" t="str">
+        <v>http://qudt.org/vocab/unit/M|http://qudt.org/vocab/unit/MegaW</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
       </c>
       <c r="B27" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C27" t="str">
-        <v>Een typering van verschillende procedures.</v>
+        <v>null</v>
       </c>
       <c r="D27" t="str">
         <v>null</v>
       </c>
       <c r="E27" t="str">
-        <v>null</v>
+        <v>Emissiepunt eigenschappen</v>
       </c>
       <c r="F27" t="str">
-        <v>Een typering van verschillende procedures.</v>
+        <v>null</v>
       </c>
       <c r="G27" t="str">
-        <v>Procedure types</v>
+        <v>null</v>
       </c>
       <c r="H27" t="str">
         <v>null</v>
@@ -1728,10 +1884,10 @@
         <v>null</v>
       </c>
       <c r="J27" t="str">
-        <v>null</v>
+        <v>Een typering van verschillende eigenschappen voor emissiepunten.</v>
       </c>
       <c r="K27" t="str">
-        <v>null</v>
+        <v>Een typering van verschillende eigenschappen voor emissiepunten.</v>
       </c>
       <c r="L27" t="str">
         <v>null</v>
@@ -1743,33 +1899,39 @@
         <v>null</v>
       </c>
       <c r="O27" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/emissie|https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/onttrekking|https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/transport|https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/verwerking</v>
+        <v>null</v>
       </c>
       <c r="P27" t="str">
         <v>null</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>null</v>
+      </c>
+      <c r="R27" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/schouw-diameter|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/schouw-hoogte</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_type</v>
       </c>
       <c r="B28" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C28" t="str">
-        <v>Een typering van verschillende statussen (actief, inactief, ...).</v>
+        <v>null</v>
       </c>
       <c r="D28" t="str">
         <v>null</v>
       </c>
       <c r="E28" t="str">
-        <v>null</v>
+        <v>Emissiepunt types</v>
       </c>
       <c r="F28" t="str">
-        <v>Een typering van verschillende statussen (actief, inactief, ...).</v>
+        <v>null</v>
       </c>
       <c r="G28" t="str">
-        <v>Status types</v>
+        <v>null</v>
       </c>
       <c r="H28" t="str">
         <v>null</v>
@@ -1778,10 +1940,10 @@
         <v>null</v>
       </c>
       <c r="J28" t="str">
-        <v>null</v>
+        <v>Een typering van verschillende soorten emissiepunten.</v>
       </c>
       <c r="K28" t="str">
-        <v>null</v>
+        <v>Een typering van verschillende soorten emissiepunten.</v>
       </c>
       <c r="L28" t="str">
         <v>null</v>
@@ -1793,45 +1955,51 @@
         <v>null</v>
       </c>
       <c r="O28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/definitief_uit_dienst|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/in_dienst|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/ontmanteld|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/tijdelijk_uit_dienst|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/voorgesteld</v>
+        <v>null</v>
       </c>
       <c r="P28" t="str">
         <v>null</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>null</v>
+      </c>
+      <c r="R28" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schouw|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/emissiepunt|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/lozingspunt|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_vertikale_uitstroom</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>riepr-emissiepunt-eigenschappen:schouw-diameter</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_eigenschappen</v>
       </c>
       <c r="B29" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C29" t="str">
         <v>null</v>
       </c>
       <c r="D29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
+        <v>null</v>
       </c>
       <c r="E29" t="str">
-        <v>diameter</v>
+        <v>Installatie eigenschappen</v>
       </c>
       <c r="F29" t="str">
         <v>null</v>
       </c>
       <c r="G29" t="str">
-        <v>Diameter van de schouw</v>
+        <v>null</v>
       </c>
       <c r="H29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
+        <v>null</v>
       </c>
       <c r="I29" t="str">
         <v>null</v>
       </c>
       <c r="J29" t="str">
-        <v>null</v>
+        <v>Een typering van verschillende eigenschappen voor installaties.</v>
       </c>
       <c r="K29" t="str">
-        <v>null</v>
+        <v>Een typering van verschillende eigenschappen voor installaties.</v>
       </c>
       <c r="L29" t="str">
         <v>null</v>
@@ -1846,42 +2014,48 @@
         <v>null</v>
       </c>
       <c r="P29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schouw</v>
+        <v>null</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>null</v>
+      </c>
+      <c r="R29" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerd_vermogen</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>riepr-emissiepunt-eigenschappen:schouw-hoogte</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_type</v>
       </c>
       <c r="B30" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C30" t="str">
         <v>null</v>
       </c>
       <c r="D30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
+        <v>null</v>
       </c>
       <c r="E30" t="str">
-        <v>hoogte</v>
+        <v>Installatie types</v>
       </c>
       <c r="F30" t="str">
         <v>null</v>
       </c>
       <c r="G30" t="str">
-        <v>Hoogte van de schouw</v>
+        <v>null</v>
       </c>
       <c r="H30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/emissiepunt_eigenschappen</v>
+        <v>null</v>
       </c>
       <c r="I30" t="str">
         <v>null</v>
       </c>
       <c r="J30" t="str">
-        <v>null</v>
+        <v>Een typering van verschillende soorten installaties.</v>
       </c>
       <c r="K30" t="str">
-        <v>null</v>
+        <v>Een typering van verschillende soorten installaties.</v>
       </c>
       <c r="L30" t="str">
         <v>null</v>
@@ -1896,33 +2070,39 @@
         <v>null</v>
       </c>
       <c r="P30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schouw</v>
+        <v>null</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>null</v>
+      </c>
+      <c r="R30" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>riepr-installatie-eigenschappen:geinstalleerd_vermogen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/meetpunt_type</v>
       </c>
       <c r="B31" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C31" t="str">
         <v>null</v>
       </c>
       <c r="D31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_eigenschappen</v>
+        <v>null</v>
       </c>
       <c r="E31" t="str">
-        <v>GEINSTALLEERD_VERMOGEN</v>
+        <v>Meetpunt types</v>
       </c>
       <c r="F31" t="str">
         <v>null</v>
       </c>
       <c r="G31" t="str">
-        <v>Geinstalleerd vermogen</v>
+        <v>null</v>
       </c>
       <c r="H31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/installatie_eigenschappen</v>
+        <v>null</v>
       </c>
       <c r="I31" t="str">
         <v>null</v>
@@ -1946,12 +2126,186 @@
         <v>null</v>
       </c>
       <c r="P31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie</v>
+        <v>null</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>null</v>
+      </c>
+      <c r="R31" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/meetput</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/onttrekkingspunt_type</v>
+      </c>
+      <c r="B32" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+      </c>
+      <c r="C32" t="str">
+        <v>null</v>
+      </c>
+      <c r="D32" t="str">
+        <v>null</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Onttrekkingspunt types</v>
+      </c>
+      <c r="F32" t="str">
+        <v>null</v>
+      </c>
+      <c r="G32" t="str">
+        <v>null</v>
+      </c>
+      <c r="H32" t="str">
+        <v>null</v>
+      </c>
+      <c r="I32" t="str">
+        <v>null</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Een typering van verschillende soorten onttrekkingspunten.</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Een typering van verschillende soorten onttrekkingspunten.</v>
+      </c>
+      <c r="L32" t="str">
+        <v>null</v>
+      </c>
+      <c r="M32" t="str">
+        <v>null</v>
+      </c>
+      <c r="N32" t="str">
+        <v>null</v>
+      </c>
+      <c r="O32" t="str">
+        <v>null</v>
+      </c>
+      <c r="P32" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>null</v>
+      </c>
+      <c r="R32" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-type/grondwaterput</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/procedure_type</v>
+      </c>
+      <c r="B33" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+      </c>
+      <c r="C33" t="str">
+        <v>null</v>
+      </c>
+      <c r="D33" t="str">
+        <v>null</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Procedure types</v>
+      </c>
+      <c r="F33" t="str">
+        <v>null</v>
+      </c>
+      <c r="G33" t="str">
+        <v>null</v>
+      </c>
+      <c r="H33" t="str">
+        <v>null</v>
+      </c>
+      <c r="I33" t="str">
+        <v>null</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Een typering van verschillende procedures.</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Een typering van verschillende procedures.</v>
+      </c>
+      <c r="L33" t="str">
+        <v>null</v>
+      </c>
+      <c r="M33" t="str">
+        <v>null</v>
+      </c>
+      <c r="N33" t="str">
+        <v>null</v>
+      </c>
+      <c r="O33" t="str">
+        <v>null</v>
+      </c>
+      <c r="P33" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>null</v>
+      </c>
+      <c r="R33" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/emissie|https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/onttrekking|https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/transport|https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/verwerking</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/status_type</v>
+      </c>
+      <c r="B34" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+      </c>
+      <c r="C34" t="str">
+        <v>null</v>
+      </c>
+      <c r="D34" t="str">
+        <v>null</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Status types</v>
+      </c>
+      <c r="F34" t="str">
+        <v>null</v>
+      </c>
+      <c r="G34" t="str">
+        <v>null</v>
+      </c>
+      <c r="H34" t="str">
+        <v>null</v>
+      </c>
+      <c r="I34" t="str">
+        <v>null</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Een typering van verschillende statussen (actief, inactief, ...).</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Een typering van verschillende statussen (actief, inactief, ...).</v>
+      </c>
+      <c r="L34" t="str">
+        <v>null</v>
+      </c>
+      <c r="M34" t="str">
+        <v>null</v>
+      </c>
+      <c r="N34" t="str">
+        <v>null</v>
+      </c>
+      <c r="O34" t="str">
+        <v>null</v>
+      </c>
+      <c r="P34" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>null</v>
+      </c>
+      <c r="R34" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/definitief_uit_dienst|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/in_dienst|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/ontmanteld|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/tijdelijk_uit_dienst|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/voorgesteld</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: verplicht en meervoudig
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/rie-iepr/rie-iepr.xlsx
+++ b/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/rie-iepr/rie-iepr.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S45"/>
+  <dimension ref="A1:U45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,12 +449,18 @@
         <v>broaderTransitive</v>
       </c>
       <c r="Q1" t="str">
+        <v>isVerplicht</v>
+      </c>
+      <c r="R1" t="str">
+        <v>isMeervoudig</v>
+      </c>
+      <c r="S1" t="str">
         <v>parameterDimensie</v>
       </c>
-      <c r="R1" t="str">
+      <c r="T1" t="str">
         <v>seeAlso</v>
       </c>
-      <c r="S1" t="str">
+      <c r="U1" t="str">
         <v>hasTopConcept</v>
       </c>
     </row>
@@ -516,6 +522,12 @@
       <c r="S2" t="str">
         <v>null</v>
       </c>
+      <c r="T2" t="str">
+        <v>null</v>
+      </c>
+      <c r="U2" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -575,6 +587,12 @@
       <c r="S3" t="str">
         <v>null</v>
       </c>
+      <c r="T3" t="str">
+        <v>null</v>
+      </c>
+      <c r="U3" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -634,6 +652,12 @@
       <c r="S4" t="str">
         <v>null</v>
       </c>
+      <c r="T4" t="str">
+        <v>null</v>
+      </c>
+      <c r="U4" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -693,6 +717,12 @@
       <c r="S5" t="str">
         <v>null</v>
       </c>
+      <c r="T5" t="str">
+        <v>null</v>
+      </c>
+      <c r="U5" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -752,6 +782,12 @@
       <c r="S6" t="str">
         <v>null</v>
       </c>
+      <c r="T6" t="str">
+        <v>null</v>
+      </c>
+      <c r="U6" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -811,6 +847,12 @@
       <c r="S7" t="str">
         <v>null</v>
       </c>
+      <c r="T7" t="str">
+        <v>null</v>
+      </c>
+      <c r="U7" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -870,6 +912,12 @@
       <c r="S8" t="str">
         <v>null</v>
       </c>
+      <c r="T8" t="str">
+        <v>null</v>
+      </c>
+      <c r="U8" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -929,6 +977,12 @@
       <c r="S9" t="str">
         <v>null</v>
       </c>
+      <c r="T9" t="str">
+        <v>null</v>
+      </c>
+      <c r="U9" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -988,6 +1042,12 @@
       <c r="S10" t="str">
         <v>null</v>
       </c>
+      <c r="T10" t="str">
+        <v>null</v>
+      </c>
+      <c r="U10" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -1047,6 +1107,12 @@
       <c r="S11" t="str">
         <v>null</v>
       </c>
+      <c r="T11" t="str">
+        <v>null</v>
+      </c>
+      <c r="U11" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1106,6 +1172,12 @@
       <c r="S12" t="str">
         <v>null</v>
       </c>
+      <c r="T12" t="str">
+        <v>null</v>
+      </c>
+      <c r="U12" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1165,6 +1237,12 @@
       <c r="S13" t="str">
         <v>null</v>
       </c>
+      <c r="T13" t="str">
+        <v>null</v>
+      </c>
+      <c r="U13" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1224,6 +1302,12 @@
       <c r="S14" t="str">
         <v>null</v>
       </c>
+      <c r="T14" t="str">
+        <v>null</v>
+      </c>
+      <c r="U14" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1283,6 +1367,12 @@
       <c r="S15" t="str">
         <v>null</v>
       </c>
+      <c r="T15" t="str">
+        <v>null</v>
+      </c>
+      <c r="U15" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1342,6 +1432,12 @@
       <c r="S16" t="str">
         <v>null</v>
       </c>
+      <c r="T16" t="str">
+        <v>null</v>
+      </c>
+      <c r="U16" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1401,6 +1497,12 @@
       <c r="S17" t="str">
         <v>null</v>
       </c>
+      <c r="T17" t="str">
+        <v>null</v>
+      </c>
+      <c r="U17" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1460,6 +1562,12 @@
       <c r="S18" t="str">
         <v>null</v>
       </c>
+      <c r="T18" t="str">
+        <v>null</v>
+      </c>
+      <c r="U18" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1519,6 +1627,12 @@
       <c r="S19" t="str">
         <v>null</v>
       </c>
+      <c r="T19" t="str">
+        <v>null</v>
+      </c>
+      <c r="U19" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1570,12 +1684,18 @@
         <v>null</v>
       </c>
       <c r="Q20" t="str">
-        <v>null</v>
+        <v>true</v>
       </c>
       <c r="R20" t="str">
         <v>null</v>
       </c>
       <c r="S20" t="str">
+        <v>null</v>
+      </c>
+      <c r="T20" t="str">
+        <v>null</v>
+      </c>
+      <c r="U20" t="str">
         <v>null</v>
       </c>
     </row>
@@ -1629,12 +1749,18 @@
         <v>null</v>
       </c>
       <c r="Q21" t="str">
+        <v>null</v>
+      </c>
+      <c r="R21" t="str">
+        <v>true</v>
+      </c>
+      <c r="S21" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/riepr/chemische_stof</v>
       </c>
-      <c r="R21" t="str">
-        <v>null</v>
-      </c>
-      <c r="S21" t="str">
+      <c r="T21" t="str">
+        <v>null</v>
+      </c>
+      <c r="U21" t="str">
         <v>null</v>
       </c>
     </row>
@@ -1696,6 +1822,12 @@
       <c r="S22" t="str">
         <v>null</v>
       </c>
+      <c r="T22" t="str">
+        <v>null</v>
+      </c>
+      <c r="U22" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1755,6 +1887,12 @@
       <c r="S23" t="str">
         <v>null</v>
       </c>
+      <c r="T23" t="str">
+        <v>null</v>
+      </c>
+      <c r="U23" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1814,6 +1952,12 @@
       <c r="S24" t="str">
         <v>null</v>
       </c>
+      <c r="T24" t="str">
+        <v>null</v>
+      </c>
+      <c r="U24" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1873,6 +2017,12 @@
       <c r="S25" t="str">
         <v>null</v>
       </c>
+      <c r="T25" t="str">
+        <v>null</v>
+      </c>
+      <c r="U25" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1932,6 +2082,12 @@
       <c r="S26" t="str">
         <v>null</v>
       </c>
+      <c r="T26" t="str">
+        <v>null</v>
+      </c>
+      <c r="U26" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1991,6 +2147,12 @@
       <c r="S27" t="str">
         <v>null</v>
       </c>
+      <c r="T27" t="str">
+        <v>null</v>
+      </c>
+      <c r="U27" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -2050,6 +2212,12 @@
       <c r="S28" t="str">
         <v>null</v>
       </c>
+      <c r="T28" t="str">
+        <v>null</v>
+      </c>
+      <c r="U28" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -2109,6 +2277,12 @@
       <c r="S29" t="str">
         <v>null</v>
       </c>
+      <c r="T29" t="str">
+        <v>null</v>
+      </c>
+      <c r="U29" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -2168,6 +2342,12 @@
       <c r="S30" t="str">
         <v>null</v>
       </c>
+      <c r="T30" t="str">
+        <v>null</v>
+      </c>
+      <c r="U30" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -2227,6 +2407,12 @@
       <c r="S31" t="str">
         <v>null</v>
       </c>
+      <c r="T31" t="str">
+        <v>null</v>
+      </c>
+      <c r="U31" t="str">
+        <v>null</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -2281,9 +2467,15 @@
         <v>null</v>
       </c>
       <c r="R32" t="str">
+        <v>null</v>
+      </c>
+      <c r="S32" t="str">
+        <v>null</v>
+      </c>
+      <c r="T32" t="str">
         <v>http://purl.org/adms/status/Withdrawn</v>
       </c>
-      <c r="S32" t="str">
+      <c r="U32" t="str">
         <v>null</v>
       </c>
     </row>
@@ -2340,9 +2532,15 @@
         <v>null</v>
       </c>
       <c r="R33" t="str">
+        <v>null</v>
+      </c>
+      <c r="S33" t="str">
+        <v>null</v>
+      </c>
+      <c r="T33" t="str">
         <v>http://purl.org/adms/status/Completed</v>
       </c>
-      <c r="S33" t="str">
+      <c r="U33" t="str">
         <v>null</v>
       </c>
     </row>
@@ -2399,9 +2597,15 @@
         <v>null</v>
       </c>
       <c r="R34" t="str">
+        <v>null</v>
+      </c>
+      <c r="S34" t="str">
+        <v>null</v>
+      </c>
+      <c r="T34" t="str">
         <v>http://purl.org/adms/status/Withdrawn</v>
       </c>
-      <c r="S34" t="str">
+      <c r="U34" t="str">
         <v>null</v>
       </c>
     </row>
@@ -2458,9 +2662,15 @@
         <v>null</v>
       </c>
       <c r="R35" t="str">
+        <v>null</v>
+      </c>
+      <c r="S35" t="str">
+        <v>null</v>
+      </c>
+      <c r="T35" t="str">
         <v>http://purl.org/adms/status/Deprecated</v>
       </c>
-      <c r="S35" t="str">
+      <c r="U35" t="str">
         <v>null</v>
       </c>
     </row>
@@ -2517,9 +2727,15 @@
         <v>null</v>
       </c>
       <c r="R36" t="str">
+        <v>null</v>
+      </c>
+      <c r="S36" t="str">
+        <v>null</v>
+      </c>
+      <c r="T36" t="str">
         <v>http://purl.org/adms/status/UnderDevelopment</v>
       </c>
-      <c r="S36" t="str">
+      <c r="U36" t="str">
         <v>null</v>
       </c>
     </row>
@@ -2579,6 +2795,12 @@
         <v>null</v>
       </c>
       <c r="S37" t="str">
+        <v>null</v>
+      </c>
+      <c r="T37" t="str">
+        <v>null</v>
+      </c>
+      <c r="U37" t="str">
         <v>http://qudt.org/vocab/unit/DEG_C|http://qudt.org/vocab/unit/K|http://qudt.org/vocab/unit/M|http://qudt.org/vocab/unit/MegaW|http://qudt.org/vocab/unit/MicroGM-PER-L|http://qudt.org/vocab/unit/MilliGM-PER-L|http://qudt.org/vocab/unit/NanoGM-PER-L|http://qudt.org/vocab/unit/PERCENT|http://qudt.org/vocab/unit/PPB|http://qudt.org/vocab/unit/PPM</v>
       </c>
     </row>
@@ -2638,6 +2860,12 @@
         <v>null</v>
       </c>
       <c r="S38" t="str">
+        <v>null</v>
+      </c>
+      <c r="T38" t="str">
+        <v>null</v>
+      </c>
+      <c r="U38" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/schouw-diameter|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-eigenschappen/schouw-hoogte</v>
       </c>
     </row>
@@ -2697,6 +2925,12 @@
         <v>null</v>
       </c>
       <c r="S39" t="str">
+        <v>null</v>
+      </c>
+      <c r="T39" t="str">
+        <v>null</v>
+      </c>
+      <c r="U39" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schouw|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/emissiepunt|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/lozingspunt|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_horizontale_uitstroom|https://data.omgeving.vlaanderen.be/id/concept/riepr/emissiepunt-type/schoorsteen_verticale_uitstroom</v>
       </c>
     </row>
@@ -2756,6 +2990,12 @@
         <v>null</v>
       </c>
       <c r="S40" t="str">
+        <v>null</v>
+      </c>
+      <c r="T40" t="str">
+        <v>null</v>
+      </c>
+      <c r="U40" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/geinstalleerd_vermogen|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-eigenschappen/verwijderingsrendement</v>
       </c>
     </row>
@@ -2815,6 +3055,12 @@
         <v>null</v>
       </c>
       <c r="S41" t="str">
+        <v>null</v>
+      </c>
+      <c r="T41" t="str">
+        <v>null</v>
+      </c>
+      <c r="U41" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/stookinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/filterinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/directe_stookinstallatie|https://data.omgeving.vlaanderen.be/id/concept/riepr/installatie-type/installatie</v>
       </c>
     </row>
@@ -2874,6 +3120,12 @@
         <v>null</v>
       </c>
       <c r="S42" t="str">
+        <v>null</v>
+      </c>
+      <c r="T42" t="str">
+        <v>null</v>
+      </c>
+      <c r="U42" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/meetpunt-type/meetput</v>
       </c>
     </row>
@@ -2933,6 +3185,12 @@
         <v>null</v>
       </c>
       <c r="S43" t="str">
+        <v>null</v>
+      </c>
+      <c r="T43" t="str">
+        <v>null</v>
+      </c>
+      <c r="U43" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/onttrekkingspunt-type/grondwaterput</v>
       </c>
     </row>
@@ -2992,6 +3250,12 @@
         <v>null</v>
       </c>
       <c r="S44" t="str">
+        <v>null</v>
+      </c>
+      <c r="T44" t="str">
+        <v>null</v>
+      </c>
+      <c r="U44" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/emissie|https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/onttrekking|https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/transport|https://data.omgeving.vlaanderen.be/id/concept/riepr/procedure-type/verwerking</v>
       </c>
     </row>
@@ -3051,12 +3315,18 @@
         <v>null</v>
       </c>
       <c r="S45" t="str">
+        <v>null</v>
+      </c>
+      <c r="T45" t="str">
+        <v>null</v>
+      </c>
+      <c r="U45" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/definitief_uit_dienst|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/in_dienst|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/ontmanteld|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/tijdelijk_uit_dienst|https://data.omgeving.vlaanderen.be/id/concept/riepr/status-type/voorgesteld</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U45"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>